<commit_message>
Make the linear regression walkthrough dataset reproduce both demos
</commit_message>
<xml_diff>
--- a/lesson2-advanced-data-analysis/linear-regression-walkthrough.xlsx
+++ b/lesson2-advanced-data-analysis/linear-regression-walkthrough.xlsx
@@ -316,7 +316,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>54900</v>
+        <v>53318</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -324,7 +324,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1">
-        <v>54300</v>
+        <v>53061</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -332,7 +332,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>54150</v>
+        <v>52997</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -340,7 +340,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="1">
-        <v>53976</v>
+        <v>52923</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -348,7 +348,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="1">
-        <v>53723</v>
+        <v>52814</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -356,7 +356,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="1">
-        <v>53580</v>
+        <v>52753</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -364,7 +364,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="1">
-        <v>53443</v>
+        <v>52694</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -372,7 +372,7 @@
         <v>0</v>
       </c>
       <c r="B9" s="1">
-        <v>53395</v>
+        <v>52674</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -380,7 +380,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="1">
-        <v>52997</v>
+        <v>52504</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -388,7 +388,7 @@
         <v>0</v>
       </c>
       <c r="B11" s="1">
-        <v>52853</v>
+        <v>52442</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -396,7 +396,7 @@
         <v>0</v>
       </c>
       <c r="B12" s="1">
-        <v>52293</v>
+        <v>52202</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -404,7 +404,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="1">
-        <v>52211</v>
+        <v>52167</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -412,7 +412,7 @@
         <v>0</v>
       </c>
       <c r="B14" s="1">
-        <v>52143</v>
+        <v>52138</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -420,7 +420,7 @@
         <v>0</v>
       </c>
       <c r="B15" s="1">
-        <v>52086</v>
+        <v>52114</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -428,7 +428,7 @@
         <v>0</v>
       </c>
       <c r="B16" s="1">
-        <v>51871</v>
+        <v>52022</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -436,7 +436,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="1">
-        <v>51839</v>
+        <v>52008</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -444,7 +444,7 @@
         <v>0</v>
       </c>
       <c r="B18" s="1">
-        <v>51511</v>
+        <v>51868</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -452,7 +452,7 @@
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>51259</v>
+        <v>51760</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -460,7 +460,7 @@
         <v>0</v>
       </c>
       <c r="B20" s="1">
-        <v>50954</v>
+        <v>51629</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -468,7 +468,7 @@
         <v>0</v>
       </c>
       <c r="B21" s="1">
-        <v>50894</v>
+        <v>51604</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -476,7 +476,7 @@
         <v>0</v>
       </c>
       <c r="B22" s="1">
-        <v>50666</v>
+        <v>51506</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -484,7 +484,7 @@
         <v>0</v>
       </c>
       <c r="B23" s="1">
-        <v>50499</v>
+        <v>51435</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -492,7 +492,7 @@
         <v>0</v>
       </c>
       <c r="B24" s="1">
-        <v>50497</v>
+        <v>51434</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -500,7 +500,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B25" s="1">
-        <v>53354</v>
+        <v>52142</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -508,7 +508,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B26" s="1">
-        <v>53314</v>
+        <v>52125</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -516,7 +516,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B27" s="1">
-        <v>53286</v>
+        <v>52113</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -524,7 +524,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B28" s="1">
-        <v>52806</v>
+        <v>51908</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -532,7 +532,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B29" s="1">
-        <v>52372</v>
+        <v>51722</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -540,7 +540,7 @@
         <v>6.6669999999999993E-2</v>
       </c>
       <c r="B30" s="1">
-        <v>49358</v>
+        <v>50432</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -548,7 +548,7 @@
         <v>0.1</v>
       </c>
       <c r="B31" s="1">
-        <v>52691</v>
+        <v>51602</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -556,7 +556,7 @@
         <v>0.1</v>
       </c>
       <c r="B32" s="1">
-        <v>52539</v>
+        <v>51536</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -564,7 +564,7 @@
         <v>0.1</v>
       </c>
       <c r="B33" s="1">
-        <v>51844</v>
+        <v>51239</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -572,7 +572,7 @@
         <v>0.1</v>
       </c>
       <c r="B34" s="1">
-        <v>51588</v>
+        <v>51129</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -580,7 +580,7 @@
         <v>0.1</v>
       </c>
       <c r="B35" s="1">
-        <v>51141</v>
+        <v>50938</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -588,7 +588,7 @@
         <v>0.1</v>
       </c>
       <c r="B36" s="1">
-        <v>51015</v>
+        <v>50884</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -596,7 +596,7 @@
         <v>0.1</v>
       </c>
       <c r="B37" s="1">
-        <v>49923</v>
+        <v>50417</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -604,7 +604,7 @@
         <v>0.1</v>
       </c>
       <c r="B38" s="1">
-        <v>49521</v>
+        <v>50245</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -612,7 +612,7 @@
         <v>0.1</v>
       </c>
       <c r="B39" s="1">
-        <v>49315</v>
+        <v>50157</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -620,7 +620,7 @@
         <v>0.1</v>
       </c>
       <c r="B40" s="1">
-        <v>48625</v>
+        <v>49861</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -628,7 +628,7 @@
         <v>0.13333</v>
       </c>
       <c r="B41" s="1">
-        <v>53210</v>
+        <v>51567</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -636,7 +636,7 @@
         <v>0.13333</v>
       </c>
       <c r="B42" s="1">
-        <v>52912</v>
+        <v>51439</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -644,7 +644,7 @@
         <v>0.13333</v>
       </c>
       <c r="B43" s="1">
-        <v>52373</v>
+        <v>51208</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -652,7 +652,7 @@
         <v>0.13333</v>
       </c>
       <c r="B44" s="1">
-        <v>50788</v>
+        <v>50530</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -660,7 +660,7 @@
         <v>0.13333</v>
       </c>
       <c r="B45" s="1">
-        <v>50375</v>
+        <v>50353</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -668,7 +668,7 @@
         <v>0.13333</v>
       </c>
       <c r="B46" s="1">
-        <v>49840</v>
+        <v>50124</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -676,7 +676,7 @@
         <v>0.13333</v>
       </c>
       <c r="B47" s="1">
-        <v>49506</v>
+        <v>49981</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -684,7 +684,7 @@
         <v>0.13333</v>
       </c>
       <c r="B48" s="1">
-        <v>48428</v>
+        <v>49520</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -692,7 +692,7 @@
         <v>0.2</v>
       </c>
       <c r="B49" s="1">
-        <v>51680</v>
+        <v>50398</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -700,7 +700,7 @@
         <v>0.2</v>
       </c>
       <c r="B50" s="1">
-        <v>50451</v>
+        <v>49872</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -708,7 +708,7 @@
         <v>0.2</v>
       </c>
       <c r="B51" s="1">
-        <v>50109</v>
+        <v>49725</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -716,7 +716,7 @@
         <v>0.2</v>
       </c>
       <c r="B52" s="1">
-        <v>49337</v>
+        <v>49395</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -724,7 +724,7 @@
         <v>0.2</v>
       </c>
       <c r="B53" s="1">
-        <v>49312</v>
+        <v>49384</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -732,7 +732,7 @@
         <v>0.2</v>
       </c>
       <c r="B54" s="1">
-        <v>49179</v>
+        <v>49327</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -740,7 +740,7 @@
         <v>0.2</v>
       </c>
       <c r="B55" s="1">
-        <v>48701</v>
+        <v>49123</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -748,7 +748,7 @@
         <v>0.2</v>
       </c>
       <c r="B56" s="1">
-        <v>48675</v>
+        <v>49112</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -756,7 +756,7 @@
         <v>0.2</v>
       </c>
       <c r="B57" s="1">
-        <v>48360</v>
+        <v>48977</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -764,7 +764,7 @@
         <v>0.25</v>
       </c>
       <c r="B58" s="1">
-        <v>49440</v>
+        <v>49054</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -772,7 +772,7 @@
         <v>0.25</v>
       </c>
       <c r="B59" s="1">
-        <v>48892</v>
+        <v>48819</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -780,7 +780,7 @@
         <v>0.35</v>
       </c>
       <c r="B60" s="1">
-        <v>45274</v>
+        <v>46500</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -788,7 +788,7 @@
         <v>0.5</v>
       </c>
       <c r="B61" s="1">
-        <v>44595</v>
+        <v>45052</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -796,7 +796,7 @@
         <v>0.75</v>
       </c>
       <c r="B62" s="1">
-        <v>42104</v>
+        <v>42059</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -804,7 +804,7 @@
         <v>0.75</v>
       </c>
       <c r="B63" s="1">
-        <v>40796</v>
+        <v>41499</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -812,7 +812,7 @@
         <v>0.84</v>
       </c>
       <c r="B64" s="1">
-        <v>37748</v>
+        <v>39500</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -820,7 +820,7 @@
         <v>0.9</v>
       </c>
       <c r="B65" s="1">
-        <v>38486</v>
+        <v>39354</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -828,7 +828,7 @@
         <v>1.25</v>
       </c>
       <c r="B66" s="1">
-        <v>38921</v>
+        <v>36840</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -836,7 +836,7 @@
         <v>1.25</v>
       </c>
       <c r="B67" s="1">
-        <v>34728</v>
+        <v>35047</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -844,7 +844,7 @@
         <v>1.25</v>
       </c>
       <c r="B68" s="1">
-        <v>33369</v>
+        <v>34465</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -852,7 +852,7 @@
         <v>1.25</v>
       </c>
       <c r="B69" s="1">
-        <v>31039</v>
+        <v>33468</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
@@ -860,7 +860,7 @@
         <v>1.25</v>
       </c>
       <c r="B70" s="1">
-        <v>27259</v>
+        <v>31850</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -868,7 +868,7 @@
         <v>0.72509999999999997</v>
       </c>
       <c r="B71">
-        <v>39524</v>
+        <v>40936</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -876,7 +876,7 @@
         <v>0.72509999999999997</v>
       </c>
       <c r="B72">
-        <v>39524</v>
+        <v>41080</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -884,7 +884,7 @@
         <v>0.72509999999999997</v>
       </c>
       <c r="B73">
-        <v>39524</v>
+        <v>41250</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -892,7 +892,7 @@
         <v>0.72509999999999997</v>
       </c>
       <c r="B74">
-        <v>39524</v>
+        <v>41322</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="B75">
-        <v>42567</v>
+        <v>47957</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -908,7 +908,7 @@
         <v>0</v>
       </c>
       <c r="B76">
-        <v>42567</v>
+        <v>48123</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -916,7 +916,7 @@
         <v>0.9</v>
       </c>
       <c r="B77">
-        <v>54755</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -924,7 +924,7 @@
         <v>0.9</v>
       </c>
       <c r="B78">
-        <v>54755</v>
+        <v>46399</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>